<commit_message>
Removed all test resferences. Rebuilt Doc. Added skeleton doc for Performance and Security. Updated the v1 spreadsheet
</commit_message>
<xml_diff>
--- a/v1_release_actions.xlsx
+++ b/v1_release_actions.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\utaf3\cast\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\utaf4\cast\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8911F3C6-68BB-4C61-9A08-D7A76CB3243B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03EF4419-396A-4260-BF38-244C92115297}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="465" yWindow="1710" windowWidth="26160" windowHeight="11295" xr2:uid="{9DB52CD6-C748-4526-A8A0-CAA4BE7B6362}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="59">
   <si>
     <t>Task</t>
   </si>
@@ -203,6 +203,18 @@
   </si>
   <si>
     <t>Yes</t>
+  </si>
+  <si>
+    <t>We need to define the code merge process</t>
+  </si>
+  <si>
+    <t>We may want to remove the autorefresh button (especially if a new UI is being deployed)</t>
+  </si>
+  <si>
+    <t>Remove Compilation Warnings</t>
+  </si>
+  <si>
+    <t>As many as we can</t>
   </si>
 </sst>
 </file>
@@ -282,47 +294,21 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="8">
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-      </font>
-      <alignment textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-      </font>
-      <alignment textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -401,6 +387,32 @@
       </font>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+      </font>
+      <alignment textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+      </font>
+      <alignment textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -415,15 +427,15 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{345856AE-2A30-44B9-BD64-B69ADF921A58}" name="Table1" displayName="Table1" ref="A1:F22" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0">
-  <autoFilter ref="A1:F22" xr:uid="{345856AE-2A30-44B9-BD64-B69ADF921A58}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{345856AE-2A30-44B9-BD64-B69ADF921A58}" name="Table1" displayName="Table1" ref="A1:F25" totalsRowShown="0" headerRowDxfId="7" dataDxfId="6">
+  <autoFilter ref="A1:F25" xr:uid="{345856AE-2A30-44B9-BD64-B69ADF921A58}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{4767FA67-4EB9-4C9D-935A-4981DF7B651C}" name="Task" dataDxfId="7"/>
-    <tableColumn id="2" xr3:uid="{EFB10F7A-0FAD-445F-8201-689A64A71587}" name="Notes" dataDxfId="6"/>
-    <tableColumn id="3" xr3:uid="{8D23DB5B-9B90-4A2D-B2CE-E60459E65E95}" name="Suggested assignment" dataDxfId="5"/>
-    <tableColumn id="4" xr3:uid="{A35BBADF-4830-498D-917B-526B8DBFE944}" name="Status" dataDxfId="4"/>
-    <tableColumn id="5" xr3:uid="{881CF4BB-6C1F-4C14-89DB-485AE3F69C89}" name="Priority" dataDxfId="3"/>
-    <tableColumn id="6" xr3:uid="{4602C1C0-CB96-45AE-9320-853C00CCAD88}" name="Required for v1?" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{4767FA67-4EB9-4C9D-935A-4981DF7B651C}" name="Task" dataDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{EFB10F7A-0FAD-445F-8201-689A64A71587}" name="Notes" dataDxfId="4"/>
+    <tableColumn id="3" xr3:uid="{8D23DB5B-9B90-4A2D-B2CE-E60459E65E95}" name="Suggested assignment" dataDxfId="3"/>
+    <tableColumn id="4" xr3:uid="{A35BBADF-4830-498D-917B-526B8DBFE944}" name="Status" dataDxfId="2"/>
+    <tableColumn id="5" xr3:uid="{881CF4BB-6C1F-4C14-89DB-485AE3F69C89}" name="Priority" dataDxfId="1"/>
+    <tableColumn id="6" xr3:uid="{4602C1C0-CB96-45AE-9320-853C00CCAD88}" name="Required for v1?" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -746,7 +758,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C255076-F7DD-418A-9674-04B09A609501}">
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="75.28515625" style="1" customWidth="1"/>
@@ -813,23 +825,23 @@
         <v>54</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
+    <row r="4" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="D4" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="E4" s="3" t="s">
+      <c r="D4" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="E4" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="7" t="s">
         <v>54</v>
       </c>
     </row>
@@ -1143,6 +1155,33 @@
       </c>
       <c r="F22" s="3" t="s">
         <v>24</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Cleanup the performance and security doc and convert to .htm. Move to Execution UI
</commit_message>
<xml_diff>
--- a/v1_release_actions.xlsx
+++ b/v1_release_actions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\utaf4\cast\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D03E4319-6CB5-4A21-95AA-41DBB9E5EDB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B9EED7E-A987-46B4-AD49-2C968752A9CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="465" yWindow="1710" windowWidth="26160" windowHeight="11295" xr2:uid="{9DB52CD6-C748-4526-A8A0-CAA4BE7B6362}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="64">
   <si>
     <t>Task</t>
   </si>
@@ -324,7 +324,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -351,8 +351,6 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1242,19 +1240,21 @@
         <v>29</v>
       </c>
     </row>
-    <row r="26" spans="1:6" ht="27" x14ac:dyDescent="0.25">
-      <c r="A26" s="1" t="s">
+    <row r="26" spans="1:6" s="8" customFormat="1" ht="27" x14ac:dyDescent="0.25">
+      <c r="A26" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="B26" s="1" t="s">
+      <c r="B26" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="C26" s="1" t="s">
+      <c r="C26" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="D26" s="14"/>
-      <c r="E26" s="14"/>
-      <c r="F26" s="14"/>
+      <c r="D26" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="E26" s="7"/>
+      <c r="F26" s="7"/>
     </row>
     <row r="27" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="9" t="s">
@@ -1264,11 +1264,11 @@
       <c r="C27" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="D27" s="15" t="s">
+      <c r="D27" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="E27" s="15"/>
-      <c r="F27" s="15"/>
+      <c r="E27" s="7"/>
+      <c r="F27" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Added Simple REST Web Listener. Takes HTTP GET calls with ClientId as Parameter
</commit_message>
<xml_diff>
--- a/v1_release_actions.xlsx
+++ b/v1_release_actions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\utaf4\cast\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B9EED7E-A987-46B4-AD49-2C968752A9CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D09A2C9-91AF-4A5D-A3F3-7FEED9905BDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="465" yWindow="1710" windowWidth="26160" windowHeight="11295" xr2:uid="{9DB52CD6-C748-4526-A8A0-CAA4BE7B6362}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="65">
   <si>
     <t>Task</t>
   </si>
@@ -230,6 +230,9 @@
   </si>
   <si>
     <t>Completed</t>
+  </si>
+  <si>
+    <t>Complete</t>
   </si>
 </sst>
 </file>
@@ -1179,20 +1182,23 @@
         <v>54</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A21" s="1" t="s">
+    <row r="21" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="B21" s="1" t="s">
+      <c r="B21" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="C21" s="1" t="s">
+      <c r="C21" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="E21" s="3" t="s">
+      <c r="D21" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="E21" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="F21" s="3" t="s">
+      <c r="F21" s="7" t="s">
         <v>24</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Added Client call to retrieve the UUID. Updated all of the Docs. Created new Client libraries
</commit_message>
<xml_diff>
--- a/v1_release_actions.xlsx
+++ b/v1_release_actions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\utaf4\cast\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D09A2C9-91AF-4A5D-A3F3-7FEED9905BDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E494C04B-B7DE-4686-A46D-F33FCC93B18F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="465" yWindow="1710" windowWidth="26160" windowHeight="11295" xr2:uid="{9DB52CD6-C748-4526-A8A0-CAA4BE7B6362}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="65">
   <si>
     <t>Task</t>
   </si>
@@ -1186,9 +1186,7 @@
       <c r="A21" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="B21" s="9" t="s">
-        <v>48</v>
-      </c>
+      <c r="B21" s="9"/>
       <c r="C21" s="9" t="s">
         <v>29</v>
       </c>

</xml_diff>